<commit_message>
add translations & update scripts 936e006184c4e67408ce91279b0b2e52d19d3e51
</commit_message>
<xml_diff>
--- a/nr-test-template-2/ig/StructureDefinition-cds-organization.xlsx
+++ b/nr-test-template-2/ig/StructureDefinition-cds-organization.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-06T09:36:59+00:00</t>
+    <t>2026-05-27T15:38:19+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1920,7 +1920,7 @@
     <t>Secteurs d'activité des établissements avec la même activité dans le RASS</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J101-SecteurActivite-RASS/FHIR/JDV-J101-SecteurActivite-RASS|20250828120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J101-SecteurActivite-RASS/FHIR/JDV-J101-SecteurActivite-RASS|20260223120000</t>
   </si>
   <si>
     <t>EntiteGeographique.secteurActivite</t>
@@ -1983,7 +1983,7 @@
     <t>Catégorie d'établissement du RASS</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J129-CategorieEtablissement-RASS/FHIR/JDV-J129-CategorieEtablissement-RASS|20241025120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J129-CategorieEtablissement-RASS/FHIR/JDV-J129-CategorieEtablissement-RASS|20260223120000</t>
   </si>
   <si>
     <t>EntiteGeographique.categorieEtablissement</t>
@@ -2032,7 +2032,7 @@
 Plus précisément, on distingue le code APET pour les EG (Synonyme : codeAPEN).</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J99-InseeNAFrav2Niveau5-RASS/FHIR/JDV-J99-InseeNAFrav2Niveau5-RASS|20200424120000</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J99-InseeNAFrav2Niveau5-RASS/FHIR/JDV-J99-InseeNAFrav2Niveau5-RASS|20260223120000</t>
   </si>
   <si>
     <t>EntiteJuridique.codeAPEN</t>

</xml_diff>